<commit_message>
subo actualizacion ejercicio tienda de deportes.xlsx Estadistica EXCEL
</commit_message>
<xml_diff>
--- a/estadistica-ejercicio-finde/tienda_de_deportes.xlsx
+++ b/estadistica-ejercicio-finde/tienda_de_deportes.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\curso_big_data_paula\ejercicio_rombo_y_estadistica_excel\estadistica-ejercicio-finde\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4FA0D7-EBB3-47E9-BC11-A96FD64F5275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B6E9432-974C-4068-9FD7-6C4D6BA76610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="624" yWindow="852" windowWidth="29952" windowHeight="15708" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
     <sheet name="Tabla 1" sheetId="4" r:id="rId3"/>
-    <sheet name="Ciudades" sheetId="3" r:id="rId4"/>
+    <sheet name="Canal" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="DatosExternos_1" localSheetId="2" hidden="1">'Tabla 1'!$A$1:$A$54</definedName>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="88">
   <si>
     <t>ID_Venta</t>
   </si>
@@ -299,6 +299,21 @@
   </si>
   <si>
     <t>Canal</t>
+  </si>
+  <si>
+    <t>Valoración</t>
+  </si>
+  <si>
+    <t>Tienda Física</t>
+  </si>
+  <si>
+    <t>Web</t>
+  </si>
+  <si>
+    <t>App</t>
+  </si>
+  <si>
+    <t>Promociones</t>
   </si>
 </sst>
 </file>
@@ -306,10 +321,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="167" formatCode="d\-m\-yyyy;@"/>
-    <numFmt numFmtId="168" formatCode="#,##0.00\ _€"/>
+    <numFmt numFmtId="164" formatCode="d\-m\-yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00\ _€"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,21 +332,50 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color theme="5"/>
+      </left>
+      <right style="double">
+        <color theme="5"/>
+      </right>
+      <top style="double">
+        <color theme="5"/>
+      </top>
+      <bottom style="double">
+        <color theme="5"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -340,14 +384,453 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="53">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -428,7 +911,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CAFDF4D0-7D8A-4D51-B727-588581D64311}" name="Tabla_1" displayName="Tabla_1" ref="A1:A54" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:A54" xr:uid="{CAFDF4D0-7D8A-4D51-B727-588581D64311}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{EE1EA92D-9B56-411D-81BF-754F690E1EFD}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{EE1EA92D-9B56-411D-81BF-754F690E1EFD}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -697,7 +1180,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -705,37 +1188,42 @@
     <col min="3" max="3" width="30.77734375" customWidth="1"/>
     <col min="4" max="4" width="25.21875" customWidth="1"/>
     <col min="5" max="5" width="11.77734375" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="18.44140625" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" s="3" customFormat="1" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I1" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -757,8 +1245,14 @@
       <c r="G2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -781,13 +1275,19 @@
       <c r="G3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <f t="shared" ref="B4:B19" si="0">B3+2</f>
+        <f t="shared" ref="B4:B18" si="0">B3+2</f>
         <v>45370</v>
       </c>
       <c r="C4" t="s">
@@ -805,8 +1305,14 @@
       <c r="G4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H4" t="s">
+        <v>84</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -829,8 +1335,14 @@
       <c r="G5" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H5" t="s">
+        <v>85</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -853,8 +1365,14 @@
       <c r="G6" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H6" t="s">
+        <v>84</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -877,8 +1395,14 @@
       <c r="G7" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -893,7 +1417,7 @@
         <v>18</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" s="2">
         <v>14.5</v>
@@ -901,8 +1425,14 @@
       <c r="G8" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -925,8 +1455,14 @@
       <c r="G9" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H9" t="s">
+        <v>85</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -949,8 +1485,14 @@
       <c r="G10" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H10" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -973,8 +1515,14 @@
       <c r="G11" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H11" t="s">
+        <v>84</v>
+      </c>
+      <c r="I11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -997,8 +1545,14 @@
       <c r="G12" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H12" t="s">
+        <v>85</v>
+      </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1021,8 +1575,14 @@
       <c r="G13" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H13" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1045,8 +1605,14 @@
       <c r="G14" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H14" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1069,8 +1635,14 @@
       <c r="G15" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H15" t="s">
+        <v>87</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1093,8 +1665,14 @@
       <c r="G16" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H16" t="s">
+        <v>84</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1117,8 +1695,14 @@
       <c r="G17" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H17" t="s">
+        <v>85</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1141,34 +1725,54 @@
       <c r="G18" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H18" t="s">
+        <v>84</v>
+      </c>
+      <c r="I18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B19" s="1"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D18">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
       <formula>"Electrónica"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Accesorios">
+    <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="Accesorios">
       <formula>NOT(ISERROR(SEARCH("Accesorios",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="Ropa">
+    <cfRule type="containsText" dxfId="9" priority="9" operator="containsText" text="Ropa">
       <formula>NOT(ISERROR(SEARCH("Ropa",D2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="Calzado">
+    <cfRule type="containsText" dxfId="8" priority="10" operator="containsText" text="Calzado">
       <formula>NOT(ISERROR(SEARCH("Calzado",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E18 F2">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+  <conditionalFormatting sqref="F2">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="lessThan">
       <formula>2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E18">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="lessThan">
+      <formula>2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I18">
+    <cfRule type="iconSet" priority="1">
+      <iconSet>
+        <cfvo type="percent" val="0"/>
+        <cfvo type="num" val="1"/>
+        <cfvo type="num" val="5"/>
+      </iconSet>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C23767BF-6B72-4E98-A52C-7B7F5252828D}">
           <x14:formula1>
             <xm:f>Hoja2!$A:$A</xm:f>
@@ -1180,6 +1784,12 @@
             <xm:f>'Tabla 1'!$A$2:$A$54</xm:f>
           </x14:formula1>
           <xm:sqref>G2:G18</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FE140AEF-3540-4038-9244-A9F1E9902029}">
+          <x14:formula1>
+            <xm:f>Canal!$A:$A</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2:H18</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1232,267 +1842,267 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="A7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="A9" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+      <c r="A11" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
+      <c r="A12" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+      <c r="A13" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
+      <c r="A14" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
+      <c r="A15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+      <c r="A16" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
+      <c r="A17" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
+      <c r="A18" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
+      <c r="A19" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
+      <c r="A20" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
+      <c r="A21" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
+      <c r="A22" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+      <c r="A23" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+      <c r="A24" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
+      <c r="A25" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="A26" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
+      <c r="A27" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
+      <c r="A28" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
+      <c r="A29" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
+      <c r="A30" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A31" s="3" t="s">
+      <c r="A31" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A32" s="3" t="s">
+      <c r="A32" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
+      <c r="A33" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="3" t="s">
+      <c r="A34" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
+      <c r="A35" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
+      <c r="A36" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" s="3" t="s">
+      <c r="A37" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" s="3" t="s">
+      <c r="A38" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
+      <c r="A39" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" s="3" t="s">
+      <c r="A40" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A41" s="3" t="s">
+      <c r="A41" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A42" s="3" t="s">
+      <c r="A42" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" s="3" t="s">
+      <c r="A43" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="3" t="s">
+      <c r="A44" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" s="3" t="s">
+      <c r="A45" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" s="3" t="s">
+      <c r="A46" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="3" t="s">
+      <c r="A47" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="3" t="s">
+      <c r="A48" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="3" t="s">
+      <c r="A49" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="3" t="s">
+      <c r="A50" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="3" t="s">
+      <c r="A51" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="3" t="s">
+      <c r="A52" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="3" t="s">
+      <c r="A53" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" s="3" t="s">
+      <c r="A54" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1506,9 +2116,30 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C2095D2-F007-4F22-A8D5-9C3216ADDEAE}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>